<commit_message>
Add one-month maturity (amounts due) report per customer
Compute each invoice's due date as invoice date + 1 month and aggregate the
unpaid amounts per customer into overdue / due-within-1-month / later buckets;
added as an Excel sheet plus per-customer and per-invoice CSVs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012CFZ5ZYfHoGA5tKQbi6mB5
</commit_message>
<xml_diff>
--- a/analysis/output/abu_hashem_sales_debt_analysis.xlsx
+++ b/analysis/output/abu_hashem_sales_debt_analysis.xlsx
@@ -9,18 +9,20 @@
   <sheets>
     <sheet name="الملخص Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="المديونية المستحقة AR" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="المناديب Salespeople" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="العملاء Customers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="الأصناف Items" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="الفواتير الصفرية Zero" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="الاستحقاق خلال شهر Due1mo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="المناديب Salespeople" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="العملاء Customers" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="الأصناف Items" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="الفواتير الصفرية Zero" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'الملخص Summary'!$A$3:$B$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'المديونية المستحقة AR'!$A$3:$I$258</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'المناديب Salespeople'!$A$3:$H$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'العملاء Customers'!$A$3:$I$113</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'الأصناف Items'!$A$3:$J$36</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'الفواتير الصفرية Zero'!$A$3:$H$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'الاستحقاق خلال شهر Due1mo'!$A$3:$J$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'المناديب Salespeople'!$A$3:$H$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'العملاء Customers'!$A$3:$I$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'الأصناف Items'!$A$3:$J$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'الفواتير الصفرية Zero'!$A$3:$H$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -8816,6 +8818,4412 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J111"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>المبالغ المستحقة لكل عميل بأجل شهر واحد (تاريخ الفاتورة + شهر) / Amounts due per customer under a one-month credit term (invoice date + 1 month)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>customer_code</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>customer</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>salesperson</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>total_due_EGP</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>overdue_EGP</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>due_within_1_month_EGP</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>due_later_EGP</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>first_due_date</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>last_due_date</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>احمد صلح المنيا</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام الصعيد</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>303659.75</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>303659.75</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>677</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>ميكس فود</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام الصعيد</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>266000.7</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>266000.7</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>729</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>حمادة شلبى</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام الصعيد</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>230214.6</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>230214.6</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>532</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>محمود العمده الصعيد</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام الصعيد</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>226945.2</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>226945.2</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>922</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>مصطفى عبدالمجيد</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام الصعيد</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>216056.6</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>216056.6</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>م اللفى</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>174553.5</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>174553.5</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>624</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>هايبر العابد</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>129975</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>129975</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>714</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>مصطفى ابو الدهب بنى سويف</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>120214.2</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>120214.2</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>962</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>الدوليه</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>هانى</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>114033</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>114033</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>884</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>ثلجه الوادي</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>90880</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>90880</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>455</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>ثلجه المهدي</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>76117.5</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>76117.5</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>918</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>مصطفى قمر بنى سويف</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام الصعيد</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>56255.25</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>56255.25</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>البوب</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>هانى</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>56008.2</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>56008.2</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>776</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>يوسف سعد الدايل مطروح</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>55351.05</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>55351.05</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>460</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>ثلجه المهندس</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="4" t="n">
+        <v>53397</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>53397</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>984</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>م القماش السماعيلية</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>48581.95</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>48581.95</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>693</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>م فوزى</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>شعبان</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="4" t="n">
+        <v>46611.6</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>46611.6</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>511</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>طارق سعيد السماعليه</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="4" t="n">
+        <v>46211.1</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>46211.1</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>974</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>احمد سمير بلطيم</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="4" t="n">
+        <v>45170</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>45170</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>772</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>تامر الغربية</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E23" s="4" t="n">
+        <v>44253</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>44253</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>802</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>شركة العل اسكندرية</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="4" t="n">
+        <v>43381.5</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>43381.5</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>328</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>ابوسليم</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="4" t="n">
+        <v>40857</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>40857</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>971</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>شركة الشريف الزقازيق</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E26" s="4" t="n">
+        <v>39060</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>39060</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>698</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>عبد الظاهر بشنيتى</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>37772</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>37772</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>المحل ابو هاشم</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>هانى</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E28" s="4" t="n">
+        <v>37606.1</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>37606.1</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>968</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>م الزينى قنا</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام الصعيد</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="4" t="n">
+        <v>35241</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>35241</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>674</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>ابو لطفى</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>شعبان</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" s="4" t="n">
+        <v>31900</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>31900</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>504</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>حدوته</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="4" t="n">
+        <v>31059</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>31059</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>786</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>م العزالى م امام</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E32" s="4" t="n">
+        <v>29309.7</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>29309.7</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>790</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة الصقر السويس</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E33" s="4" t="n">
+        <v>26304</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="3" t="n">
+        <v>26304</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>899</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>ثلجه النقيب ايمن فارس</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" s="4" t="n">
+        <v>24660</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="3" t="n">
+        <v>24660</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>975</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة الشرقاوى كفر صقر</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="4" t="n">
+        <v>21821.25</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="3" t="n">
+        <v>21821.25</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>986</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>البراهيمية فيصل</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="4" t="n">
+        <v>21174</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="3" t="n">
+        <v>21174</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>784</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>جزارة السعيد م سعيد</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="4" t="n">
+        <v>20405.25</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="3" t="n">
+        <v>20405.25</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>877</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>مطعم نور الشام</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E38" s="4" t="n">
+        <v>19994.4</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="3" t="n">
+        <v>19994.4</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>سامح توفيق</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>هانى</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="4" t="n">
+        <v>19500</v>
+      </c>
+      <c r="F39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="3" t="n">
+        <v>19500</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>955</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة مصر والسودان</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E40" s="4" t="n">
+        <v>18881.6</v>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>18881.6</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>864</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>م السوهاجى</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E41" s="4" t="n">
+        <v>18617</v>
+      </c>
+      <c r="F41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>18617</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>718</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>احمد عبود ( النور )</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E42" s="4" t="n">
+        <v>18092</v>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>18092</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>502</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>ثلجه بوجه</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="4" t="n">
+        <v>15117</v>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>15117</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>820</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>ام هايدى م بشرى</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="4" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="3" t="n">
+        <v>15000</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>561</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>احمد الرفاعي بردين</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" s="4" t="n">
+        <v>14800</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>14800</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>621</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>مطعم السوري</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E46" s="4" t="n">
+        <v>14579.6</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>14579.6</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>مطعم جدو</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>هانى</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="4" t="n">
+        <v>14130</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>14130</v>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>817</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة المهندس م سعيد</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="4" t="n">
+        <v>13805.7</v>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="3" t="n">
+        <v>13805.7</v>
+      </c>
+      <c r="H48" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>976</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>كشرى هند بلبيس</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>13800</v>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" s="3" t="n">
+        <v>13800</v>
+      </c>
+      <c r="H49" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>552</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>الحاج م عبدالعزيز بوجه</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E50" s="4" t="n">
+        <v>12755.1</v>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G50" s="3" t="n">
+        <v>12755.1</v>
+      </c>
+      <c r="H50" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>980</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>شركة الحرمين حسام حسن</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>12584.25</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="3" t="n">
+        <v>12584.25</v>
+      </c>
+      <c r="H51" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>837</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>احمد العبد شعبان</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>(غير مرتبط/unmapped)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="4" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="3" t="n">
+        <v>12000</v>
+      </c>
+      <c r="H52" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>719</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>كشرى الطيب ( النور )</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E53" s="4" t="n">
+        <v>11960</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G53" s="3" t="n">
+        <v>11960</v>
+      </c>
+      <c r="H53" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>654</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>تلجة شريف الكابتن ابو كبير</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E54" s="4" t="n">
+        <v>11527</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G54" s="3" t="n">
+        <v>11527</v>
+      </c>
+      <c r="H54" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>998</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة ابوالعز انشاص</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E55" s="4" t="n">
+        <v>11195</v>
+      </c>
+      <c r="F55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G55" s="3" t="n">
+        <v>11195</v>
+      </c>
+      <c r="H55" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>898</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>بروتين القصبجي امام</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="4" t="n">
+        <v>11194.5</v>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G56" s="3" t="n">
+        <v>11194.5</v>
+      </c>
+      <c r="H56" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>931</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>الغمراوى المقطم السوق التجارى</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E57" s="4" t="n">
+        <v>11144.25</v>
+      </c>
+      <c r="F57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" s="3" t="n">
+        <v>11144.25</v>
+      </c>
+      <c r="H57" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>985</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>هايبر ابوعمار بلبيس</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E58" s="4" t="n">
+        <v>10872.6</v>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" s="3" t="n">
+        <v>10872.6</v>
+      </c>
+      <c r="H58" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>885</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>رمضان سقارة ايمن فارس</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="4" t="n">
+        <v>10643.7</v>
+      </c>
+      <c r="F59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" s="3" t="n">
+        <v>10643.7</v>
+      </c>
+      <c r="H59" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>1007</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>مطعم لهاليبو باب الشعرية</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="4" t="n">
+        <v>10360</v>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" s="3" t="n">
+        <v>10360</v>
+      </c>
+      <c r="H60" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>738</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>م نور</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="4" t="n">
+        <v>10260</v>
+      </c>
+      <c r="F61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>10260</v>
+      </c>
+      <c r="H61" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>964</v>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة ابوجزر ابوحماد</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E62" s="4" t="n">
+        <v>9966</v>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" s="3" t="n">
+        <v>9966</v>
+      </c>
+      <c r="H62" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>438</v>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>ثلجه السيد الوكيل القرين</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="4" t="n">
+        <v>9180</v>
+      </c>
+      <c r="F63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" s="3" t="n">
+        <v>9180</v>
+      </c>
+      <c r="H63" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I63" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>887</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>محمود صبحي</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>(غير مرتبط/unmapped)</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="4" t="n">
+        <v>8564</v>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" s="3" t="n">
+        <v>8564</v>
+      </c>
+      <c r="H64" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>925</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة حور طوخ</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E65" s="4" t="n">
+        <v>7892.7</v>
+      </c>
+      <c r="F65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G65" s="3" t="n">
+        <v>7892.7</v>
+      </c>
+      <c r="H65" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I65" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>965</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة الدكتور ابوكبير</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E66" s="4" t="n">
+        <v>7840</v>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G66" s="3" t="n">
+        <v>7840</v>
+      </c>
+      <c r="H66" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>988</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>م كامل المعتمدية</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="4" t="n">
+        <v>7196.85</v>
+      </c>
+      <c r="F67" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" s="3" t="n">
+        <v>7196.85</v>
+      </c>
+      <c r="H67" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I67" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n">
+        <v>979</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة السماعيلية فاقوس</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>6820</v>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" s="3" t="n">
+        <v>6820</v>
+      </c>
+      <c r="H68" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="n">
+        <v>646</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>عبد ا عزت نصير البراء</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>6762.6</v>
+      </c>
+      <c r="F69" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" s="3" t="n">
+        <v>6762.6</v>
+      </c>
+      <c r="H69" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I69" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>940</v>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة البطل حلوان</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>6375</v>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>6375</v>
+      </c>
+      <c r="H70" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>997</v>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>عمر صلح امبابة</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E71" s="4" t="n">
+        <v>6349.2</v>
+      </c>
+      <c r="F71" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" s="3" t="n">
+        <v>6349.2</v>
+      </c>
+      <c r="H71" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J71" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="n">
+        <v>981</v>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة ارابيسك ابوكبير</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>6196.5</v>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" s="3" t="n">
+        <v>6196.5</v>
+      </c>
+      <c r="H72" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="n">
+        <v>876</v>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>مطعم الدمشقى</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E73" s="4" t="n">
+        <v>6012.8</v>
+      </c>
+      <c r="F73" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" s="3" t="n">
+        <v>6012.8</v>
+      </c>
+      <c r="H73" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="n">
+        <v>863</v>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>سيد عنتر</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>5995.2</v>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" s="3" t="n">
+        <v>5995.2</v>
+      </c>
+      <c r="H74" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="n">
+        <v>1001</v>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>منفذ امان السيدة زينيب</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="4" t="n">
+        <v>5769.85</v>
+      </c>
+      <c r="F75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" s="3" t="n">
+        <v>5769.85</v>
+      </c>
+      <c r="H75" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="n">
+        <v>999</v>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة المانة طوخ</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>5284.1</v>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" s="3" t="n">
+        <v>5284.1</v>
+      </c>
+      <c r="H76" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="n">
+        <v>915</v>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة زنين انور سلم</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E77" s="4" t="n">
+        <v>4896</v>
+      </c>
+      <c r="F77" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" s="3" t="n">
+        <v>4896</v>
+      </c>
+      <c r="H77" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="n">
+        <v>977</v>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>شركة الطويل كرداسة</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>4880</v>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" s="3" t="n">
+        <v>4880</v>
+      </c>
+      <c r="H78" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="n">
+        <v>638</v>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>مجمدات قدرى</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="4" t="n">
+        <v>4533.9</v>
+      </c>
+      <c r="F79" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" s="3" t="n">
+        <v>4533.9</v>
+      </c>
+      <c r="H79" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="J79" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="n">
+        <v>1003</v>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>رضا الجمل القلج</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>محمود السيد</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>4292</v>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" s="3" t="n">
+        <v>4292</v>
+      </c>
+      <c r="H80" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="n">
+        <v>684</v>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة الرضا</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="4" t="n">
+        <v>4049.4</v>
+      </c>
+      <c r="F81" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" s="3" t="n">
+        <v>4049.4</v>
+      </c>
+      <c r="H81" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="J81" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="n">
+        <v>1004</v>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>رضا الصعيدى حدائق القبة</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>محمود السيد</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>3996</v>
+      </c>
+      <c r="F82" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" s="3" t="n">
+        <v>3996</v>
+      </c>
+      <c r="H82" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="n">
+        <v>882</v>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>هايبر كنده شعبان</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>(غير مرتبط/unmapped)</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="4" t="n">
+        <v>3988</v>
+      </c>
+      <c r="F83" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" s="3" t="n">
+        <v>3988</v>
+      </c>
+      <c r="H83" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="J83" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="n">
+        <v>987</v>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة الجوهرة امبابة</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>3984</v>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" s="3" t="n">
+        <v>3984</v>
+      </c>
+      <c r="H84" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="n">
+        <v>643</v>
+      </c>
+      <c r="B85" s="3" t="inlineStr">
+        <is>
+          <t>منفذ بيع المنتجات الوطنية كفورنجم</t>
+        </is>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" s="4" t="n">
+        <v>3792.6</v>
+      </c>
+      <c r="F85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" s="3" t="n">
+        <v>3792.6</v>
+      </c>
+      <c r="H85" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="J85" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="n">
+        <v>923</v>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>عيسى المقطم</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>3688</v>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" s="3" t="n">
+        <v>3688</v>
+      </c>
+      <c r="H86" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>الكوثر شبين الكوم</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>هانى</t>
+        </is>
+      </c>
+      <c r="D87" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="4" t="n">
+        <v>3560</v>
+      </c>
+      <c r="F87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" s="3" t="n">
+        <v>3560</v>
+      </c>
+      <c r="H87" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="J87" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="n">
+        <v>270</v>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>سمك البر الشرقي</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>هانى</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" s="4" t="n">
+        <v>3560</v>
+      </c>
+      <c r="F88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" s="3" t="n">
+        <v>3560</v>
+      </c>
+      <c r="H88" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="n">
+        <v>978</v>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>هايبر مكة فيصل</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E89" s="4" t="n">
+        <v>3380</v>
+      </c>
+      <c r="F89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" s="3" t="n">
+        <v>3380</v>
+      </c>
+      <c r="H89" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="n">
+        <v>996</v>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>مايكل العروبة</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>3238.2</v>
+      </c>
+      <c r="F90" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" s="3" t="n">
+        <v>3238.2</v>
+      </c>
+      <c r="H90" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="n">
+        <v>991</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>ابوهاشم صفط اللبن</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" s="4" t="n">
+        <v>2880</v>
+      </c>
+      <c r="F91" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" s="3" t="n">
+        <v>2880</v>
+      </c>
+      <c r="H91" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="n">
+        <v>970</v>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة الحسن ابوحماد</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>2480</v>
+      </c>
+      <c r="F92" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" s="3" t="n">
+        <v>2480</v>
+      </c>
+      <c r="H92" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="n">
+        <v>973</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>كامل ابوسف عرب الغديرى</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" s="4" t="n">
+        <v>2377.5</v>
+      </c>
+      <c r="F93" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" s="3" t="n">
+        <v>2377.5</v>
+      </c>
+      <c r="H93" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="J93" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="n">
+        <v>982</v>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن2 السلمية</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>2331.49</v>
+      </c>
+      <c r="F94" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" s="3" t="n">
+        <v>2331.49</v>
+      </c>
+      <c r="H94" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="n">
+        <v>868</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>منفذ اسبيكو ايمن فارس</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>ايمن فارس</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="4" t="n">
+        <v>2295</v>
+      </c>
+      <c r="F95" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G95" s="3" t="n">
+        <v>2295</v>
+      </c>
+      <c r="H95" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+      <c r="J95" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>عادل دشيشة المنصورية</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" s="4" t="n">
+        <v>2071.6</v>
+      </c>
+      <c r="F96" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G96" s="3" t="n">
+        <v>2071.6</v>
+      </c>
+      <c r="H96" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I96" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J96" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="n">
+        <v>995</v>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>حسنى حسيب فيصل</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" s="4" t="n">
+        <v>2064</v>
+      </c>
+      <c r="F97" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G97" s="3" t="n">
+        <v>2064</v>
+      </c>
+      <c r="H97" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="n">
+        <v>1005</v>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>احمد بدوى سرياقوس</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>محمود السيد</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" s="4" t="n">
+        <v>1896</v>
+      </c>
+      <c r="F98" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G98" s="3" t="n">
+        <v>1896</v>
+      </c>
+      <c r="H98" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J98" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="n">
+        <v>1006</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
+        <is>
+          <t>طيبة العجوزة</t>
+        </is>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>(غير مرتبط/unmapped)</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" s="4" t="n">
+        <v>1860</v>
+      </c>
+      <c r="F99" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G99" s="3" t="n">
+        <v>1860</v>
+      </c>
+      <c r="H99" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I99" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="J99" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="n">
+        <v>963</v>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة ابودياب ابوحماد</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>حسام حسن</t>
+        </is>
+      </c>
+      <c r="D100" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="4" t="n">
+        <v>1611.85</v>
+      </c>
+      <c r="F100" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G100" s="3" t="n">
+        <v>1611.85</v>
+      </c>
+      <c r="H100" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I100" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="n">
+        <v>667</v>
+      </c>
+      <c r="B101" s="3" t="inlineStr">
+        <is>
+          <t>م العزونى</t>
+        </is>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E101" s="4" t="n">
+        <v>1524.9</v>
+      </c>
+      <c r="F101" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G101" s="3" t="n">
+        <v>1524.9</v>
+      </c>
+      <c r="H101" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I101" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="J101" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="n">
+        <v>746</v>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>ماركت م ابو مريم</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>محمد امام</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" s="4" t="n">
+        <v>1480</v>
+      </c>
+      <c r="F102" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G102" s="3" t="n">
+        <v>1480</v>
+      </c>
+      <c r="H102" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I102" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="n">
+        <v>993</v>
+      </c>
+      <c r="B103" s="3" t="inlineStr">
+        <is>
+          <t>عادل المصرى الوراق</t>
+        </is>
+      </c>
+      <c r="C103" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D103" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E103" s="4" t="n">
+        <v>1436.3</v>
+      </c>
+      <c r="F103" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G103" s="3" t="n">
+        <v>1436.3</v>
+      </c>
+      <c r="H103" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I103" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J103" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="n">
+        <v>992</v>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>الدكتور الجيزة</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E104" s="4" t="n">
+        <v>1436.3</v>
+      </c>
+      <c r="F104" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G104" s="3" t="n">
+        <v>1436.3</v>
+      </c>
+      <c r="H104" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I104" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="n">
+        <v>989</v>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>الحرمين امبابة م خليل</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" s="4" t="n">
+        <v>1380</v>
+      </c>
+      <c r="F105" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G105" s="3" t="n">
+        <v>1380</v>
+      </c>
+      <c r="H105" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I105" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="n">
+        <v>990</v>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>والى فتوح المريوطية</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>1380</v>
+      </c>
+      <c r="F106" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G106" s="3" t="n">
+        <v>1380</v>
+      </c>
+      <c r="H106" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I106" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="n">
+        <v>994</v>
+      </c>
+      <c r="B107" s="3" t="inlineStr">
+        <is>
+          <t>ثلجة الجمال فيصل</t>
+        </is>
+      </c>
+      <c r="C107" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D107" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="4" t="n">
+        <v>1179</v>
+      </c>
+      <c r="F107" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G107" s="3" t="n">
+        <v>1179</v>
+      </c>
+      <c r="H107" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I107" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="J107" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="n">
+        <v>623</v>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>الجمعيه التعاونيه الزقازيق</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>750</v>
+      </c>
+      <c r="F108" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G108" s="3" t="n">
+        <v>750</v>
+      </c>
+      <c r="H108" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I108" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="n">
+        <v>869</v>
+      </c>
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>مطعم ميكس جريل بشرى</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>محمد بشرى</t>
+        </is>
+      </c>
+      <c r="D109" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" s="4" t="n">
+        <v>683.4</v>
+      </c>
+      <c r="F109" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G109" s="3" t="n">
+        <v>683.4</v>
+      </c>
+      <c r="H109" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I109" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J109" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="n">
+        <v>1002</v>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>بوقلظ السيدة زينيب</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>محمد خليل</t>
+        </is>
+      </c>
+      <c r="D110" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" s="4" t="n">
+        <v>460</v>
+      </c>
+      <c r="F110" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G110" s="3" t="n">
+        <v>460</v>
+      </c>
+      <c r="H110" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I110" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="J110" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B111" s="3" t="inlineStr">
+        <is>
+          <t>عميل نقدى</t>
+        </is>
+      </c>
+      <c r="C111" s="3" t="inlineStr">
+        <is>
+          <t>(غير مرتبط/unmapped)</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="F111" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" s="3" t="n">
+        <v>150</v>
+      </c>
+      <c r="H111" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="J111" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:J111"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9164,7 +13572,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -12874,7 +17282,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14148,7 +18556,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>